<commit_message>
fix OLO growth rate
</commit_message>
<xml_diff>
--- a/public/olo_exp.xlsx
+++ b/public/olo_exp.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2293b72959587e28/PAYT_ANALYSIS/model/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{D30D7030-3FA5-FC45-89E7-75268989D8D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E25FB69-B7B6-7245-A531-2ECFD050CDD7}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="8_{D30D7030-3FA5-FC45-89E7-75268989D8D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4EFF69A-07F3-9546-A5AB-CAAE614B043B}"/>
   <bookViews>
     <workbookView xWindow="17720" yWindow="800" windowWidth="23400" windowHeight="23980" xr2:uid="{E219D4B1-7D27-470C-93D5-D94F3CBAEDA8}"/>
   </bookViews>
@@ -99,7 +99,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,6 +120,14 @@
       <b/>
       <sz val="10"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
@@ -161,10 +169,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -174,9 +183,11 @@
     <xf numFmtId="4" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -520,7 +531,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
@@ -529,7 +540,7 @@
     <col min="10" max="10" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -555,7 +566,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -582,7 +593,7 @@
         <v>32649039.53835969</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
@@ -613,8 +624,12 @@
         <f t="shared" si="0"/>
         <v>11393787.829113267</v>
       </c>
+      <c r="I3" s="7">
+        <f>POWER(H3/B3,1/6)-1</f>
+        <v>2.5518093612853621E-2</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
@@ -645,8 +660,12 @@
         <f t="shared" si="1"/>
         <v>10855470.576631472</v>
       </c>
+      <c r="I4" s="7">
+        <f>POWER(H4/B4,1/6)-1</f>
+        <v>2.5518093612853399E-2</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -677,8 +696,12 @@
         <f t="shared" si="1"/>
         <v>2849876.5484121931</v>
       </c>
+      <c r="I5" s="7">
+        <f>POWER(H5/B5,1/6)-1</f>
+        <v>2.5518093612853621E-2</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
@@ -709,8 +732,12 @@
         <f t="shared" si="1"/>
         <v>6512247.0847021146</v>
       </c>
+      <c r="I6" s="7">
+        <f>POWER(H6/B6,1/6)-1</f>
+        <v>2.5518093612853621E-2</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
@@ -740,6 +767,10 @@
       <c r="H7" s="6">
         <f t="shared" si="1"/>
         <v>1037657.4995006454</v>
+      </c>
+      <c r="I7" s="7">
+        <f>POWER(H7/B7,1/6)-1</f>
+        <v>2.5518093612853621E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>